<commit_message>
Lock XLSX schema · Run_Type=R1/R2 only · drop Position Stage
Final operator lock 2026-08-07 · end-of-day:
- Run_Type: R1 or R2 only (dropped _NEW suffix · freshness conveyed by
  Status color · CEO call: existing BUY green is distinct enough)
- Position Stage column DROPPED (redundant with Status · operator:
  "status/position stage is confusing")
- _runner_tag() collapsed · returns base R1/R2 always
- _rec_to_row strips any residual _NEW at write time (defensive)
- 23 historical _NEW rows stripped · 24 resulting dups deleted
- Final: 183 rows · 48 cols · Status[STRONG BUY 21, BUY 29, HOLD 101, EXIT 32]

Both markets sent · Guard 8 🟡 warnings only. Locked for the day.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/telegram/aegis_daily_2026-08-07.xlsx
+++ b/reports/telegram/aegis_daily_2026-08-07.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AEGIS Daily" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AEGIS Daily'!$A$1:$AW$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AEGIS Daily'!$A$1:$AV$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW13"/>
+  <dimension ref="A1:AV13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -463,48 +463,47 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="50" customWidth="1" min="19" max="19"/>
-    <col width="60" customWidth="1" min="20" max="20"/>
-    <col width="44" customWidth="1" min="21" max="21"/>
-    <col width="13" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
-    <col width="6" customWidth="1" min="25" max="25"/>
-    <col width="13" customWidth="1" min="26" max="26"/>
-    <col width="12" customWidth="1" min="27" max="27"/>
-    <col width="10" customWidth="1" min="28" max="28"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
+    <col width="60" customWidth="1" min="19" max="19"/>
+    <col width="44" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="6" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
     <col width="14" customWidth="1" min="29" max="29"/>
-    <col width="14" customWidth="1" min="30" max="30"/>
-    <col width="12" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
     <col width="13" customWidth="1" min="32" max="32"/>
-    <col width="13" customWidth="1" min="33" max="33"/>
-    <col width="11" customWidth="1" min="34" max="34"/>
-    <col width="9" customWidth="1" min="35" max="35"/>
-    <col width="11" customWidth="1" min="36" max="36"/>
-    <col width="8" customWidth="1" min="37" max="37"/>
-    <col width="11" customWidth="1" min="38" max="38"/>
-    <col width="8" customWidth="1" min="39" max="39"/>
-    <col width="11" customWidth="1" min="40" max="40"/>
-    <col width="13" customWidth="1" min="41" max="41"/>
-    <col width="15" customWidth="1" min="42" max="42"/>
-    <col width="12" customWidth="1" min="43" max="43"/>
-    <col width="11" customWidth="1" min="44" max="44"/>
-    <col width="32" customWidth="1" min="45" max="45"/>
-    <col width="20" customWidth="1" min="46" max="46"/>
-    <col width="18" customWidth="1" min="47" max="47"/>
-    <col width="17" customWidth="1" min="48" max="48"/>
-    <col width="20" customWidth="1" min="49" max="49"/>
+    <col width="11" customWidth="1" min="33" max="33"/>
+    <col width="9" customWidth="1" min="34" max="34"/>
+    <col width="11" customWidth="1" min="35" max="35"/>
+    <col width="8" customWidth="1" min="36" max="36"/>
+    <col width="11" customWidth="1" min="37" max="37"/>
+    <col width="8" customWidth="1" min="38" max="38"/>
+    <col width="11" customWidth="1" min="39" max="39"/>
+    <col width="13" customWidth="1" min="40" max="40"/>
+    <col width="15" customWidth="1" min="41" max="41"/>
+    <col width="12" customWidth="1" min="42" max="42"/>
+    <col width="11" customWidth="1" min="43" max="43"/>
+    <col width="32" customWidth="1" min="44" max="44"/>
+    <col width="20" customWidth="1" min="45" max="45"/>
+    <col width="18" customWidth="1" min="46" max="46"/>
+    <col width="17" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -545,210 +544,205 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Position Stage</t>
+          <t>Exit Reason</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Exit Reason</t>
+          <t>Exit P&amp;L %</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Exit P&amp;L %</t>
+          <t>Rank</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Rank</t>
+          <t>Prior Rank</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Prior Rank</t>
+          <t>Rank Δ</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Rank Δ</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Band</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Band</t>
+          <t>Risk Meter</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Risk Meter</t>
+          <t>Adj Conf</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Adj Conf</t>
+          <t>Ctx Drag</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Ctx Drag</t>
+          <t>Ctx Reason</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Ctx Reason</t>
+          <t>Story</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Story</t>
+          <t>Alerts</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Alerts</t>
+          <t>Confidence %</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Confidence %</t>
+          <t>Conf Type</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Conf Type</t>
+          <t>Model Score</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Model Score</t>
+          <t>Day</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>Trading Days</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>Trading Days</t>
+          <t>Horizon (d)</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Horizon (d)</t>
+          <t>Days Left</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>Days Left</t>
+          <t>Recommended</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>Recommended</t>
+          <t>Current Price</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>Current Price</t>
+          <t>Entry Price</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>Entry Price</t>
+          <t>Buy Zone Low</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>Buy Zone Low</t>
+          <t>Buy Zone High</t>
         </is>
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>Buy Zone High</t>
+          <t>Stop Loss</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>Stop Loss</t>
+          <t>Risk %</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
-          <t>Risk %</t>
+          <t>Target 1</t>
         </is>
       </c>
       <c r="AJ1" s="1" t="inlineStr">
         <is>
-          <t>Target 1</t>
+          <t>T1 %</t>
         </is>
       </c>
       <c r="AK1" s="1" t="inlineStr">
         <is>
-          <t>T1 %</t>
+          <t>Target 2</t>
         </is>
       </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
-          <t>Target 2</t>
+          <t>T2 %</t>
         </is>
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
-          <t>T2 %</t>
+          <t>Prev Close</t>
         </is>
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>Prev Close</t>
+          <t>Today Move %</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>Today Move %</t>
+          <t>Current Perf %</t>
         </is>
       </c>
       <c r="AP1" s="1" t="inlineStr">
         <is>
-          <t>Current Perf %</t>
+          <t>Max Gain %</t>
         </is>
       </c>
       <c r="AQ1" s="1" t="inlineStr">
         <is>
-          <t>Max Gain %</t>
+          <t>Max DD %</t>
         </is>
       </c>
       <c r="AR1" s="1" t="inlineStr">
         <is>
-          <t>Max DD %</t>
+          <t>Top Drivers</t>
         </is>
       </c>
       <c r="AS1" s="1" t="inlineStr">
         <is>
-          <t>Top Drivers</t>
+          <t>Sector</t>
         </is>
       </c>
       <c r="AT1" s="1" t="inlineStr">
         <is>
-          <t>Sector</t>
+          <t>Portfolio Weight %</t>
         </is>
       </c>
       <c r="AU1" s="1" t="inlineStr">
         <is>
-          <t>Portfolio Weight %</t>
+          <t>Expected Alpha %</t>
         </is>
       </c>
       <c r="AV1" s="1" t="inlineStr">
-        <is>
-          <t>Expected Alpha %</t>
-        </is>
-      </c>
-      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Last Updated (UTC)</t>
         </is>
@@ -790,140 +784,135 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
+      <c r="H2" s="3" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr"/>
-      <c r="J2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="K2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M2" s="3" t="n">
+        <v>79.3</v>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="Q2" s="3" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>crude +19.8% (rising) → +1.0pts · 12 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-1.0%) · Rank → 1→1 · Conf 57% · band HOLD · 14d left · → BUY</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr"/>
+      <c r="U2" s="3" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="V2" s="3" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z2" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="AA2" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="AB2" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="AC2" s="3" t="n">
+        <v>368.98</v>
+      </c>
+      <c r="AD2" s="3" t="n">
+        <v>374.36</v>
+      </c>
+      <c r="AE2" s="3" t="n">
+        <v>365.29</v>
+      </c>
+      <c r="AF2" s="3" t="n">
+        <v>372.67</v>
+      </c>
+      <c r="AG2" s="3" t="n">
+        <v>346.84</v>
+      </c>
+      <c r="AH2" s="3" t="n">
+        <v>-7.35</v>
+      </c>
+      <c r="AI2" s="3" t="n">
+        <v>413.26</v>
+      </c>
+      <c r="AJ2" s="3" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="AK2" s="3" t="n">
+        <v>457.54</v>
+      </c>
+      <c r="AL2" s="3" t="n">
+        <v>22.22</v>
+      </c>
+      <c r="AM2" s="3" t="n">
+        <v>377.15</v>
+      </c>
+      <c r="AN2" s="3" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="AO2" s="3" t="n">
+        <v>-1.44</v>
+      </c>
+      <c r="AP2" s="3" t="n">
         <v>0</v>
-      </c>
-      <c r="N2" s="3" t="n">
-        <v>79.3</v>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="P2" s="3" t="inlineStr">
-        <is>
-          <t>🟢</t>
-        </is>
-      </c>
-      <c r="Q2" s="3" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="R2" s="3" t="n">
-        <v>-0.8</v>
-      </c>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <t>crude +19.8% (rising) → +1.0pts · 12 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
-        </is>
-      </c>
-      <c r="T2" s="3" t="inlineStr">
-        <is>
-          <t>🟢 BUY (Δ-1.0%) · Rank → 1→1 · Conf 57% · band HOLD · 14d left · → BUY</t>
-        </is>
-      </c>
-      <c r="U2" s="3" t="inlineStr"/>
-      <c r="V2" s="3" t="n">
-        <v>56.8</v>
-      </c>
-      <c r="W2" s="3" t="inlineStr">
-        <is>
-          <t>Calibrated</t>
-        </is>
-      </c>
-      <c r="X2" s="3" t="n">
-        <v>29.2</v>
-      </c>
-      <c r="Y2" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="Z2" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AA2" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="AB2" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="AC2" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="AD2" s="3" t="n">
-        <v>368.98</v>
-      </c>
-      <c r="AE2" s="3" t="n">
-        <v>374.36</v>
-      </c>
-      <c r="AF2" s="3" t="n">
-        <v>365.29</v>
-      </c>
-      <c r="AG2" s="3" t="n">
-        <v>372.67</v>
-      </c>
-      <c r="AH2" s="3" t="n">
-        <v>346.84</v>
-      </c>
-      <c r="AI2" s="3" t="n">
-        <v>-7.35</v>
-      </c>
-      <c r="AJ2" s="3" t="n">
-        <v>413.26</v>
-      </c>
-      <c r="AK2" s="3" t="n">
-        <v>10.39</v>
-      </c>
-      <c r="AL2" s="3" t="n">
-        <v>457.54</v>
-      </c>
-      <c r="AM2" s="3" t="n">
-        <v>22.22</v>
-      </c>
-      <c r="AN2" s="3" t="n">
-        <v>377.15</v>
-      </c>
-      <c r="AO2" s="3" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="AP2" s="3" t="n">
-        <v>-1.44</v>
       </c>
       <c r="AQ2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AR2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS2" s="3" t="inlineStr">
+      <c r="AR2" s="3" t="inlineStr">
         <is>
           <t>Momentum · Value · Trend</t>
         </is>
       </c>
-      <c r="AT2" s="3" t="inlineStr"/>
+      <c r="AS2" s="3" t="inlineStr"/>
+      <c r="AT2" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="AU2" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV2" s="3" t="n">
         <v>10.39</v>
       </c>
-      <c r="AW2" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-07 09:51</t>
+      <c r="AV2" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:01</t>
         </is>
       </c>
     </row>
@@ -963,138 +952,133 @@
           <t>HOLD</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
+      <c r="H3" s="5" t="inlineStr"/>
       <c r="I3" s="5" t="inlineStr"/>
-      <c r="J3" s="5" t="inlineStr"/>
+      <c r="J3" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="K3" s="5" t="n">
         <v>2</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M3" s="5" t="n">
+        <v>86.5</v>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="Q3" s="5" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>crude +19.8% (rising) → +1.0pts · 5 insider Form 4 filings last 90d → +1.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>🟢 BUY (Δ-3.0%) · Rank → 2→2 · Conf 54% · band STRONG · 14d left · → HOLD</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr"/>
+      <c r="U3" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="X3" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y3" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z3" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="AA3" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="AB3" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="AC3" s="5" t="n">
+        <v>358.56</v>
+      </c>
+      <c r="AD3" s="5" t="n">
+        <v>366.13</v>
+      </c>
+      <c r="AE3" s="5" t="n">
+        <v>362.47</v>
+      </c>
+      <c r="AF3" s="5" t="n">
+        <v>369.79</v>
+      </c>
+      <c r="AG3" s="5" t="n">
+        <v>347.82</v>
+      </c>
+      <c r="AH3" s="5" t="n">
+        <v>-5</v>
+      </c>
+      <c r="AI3" s="5" t="n">
+        <v>395.42</v>
+      </c>
+      <c r="AJ3" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="AK3" s="5" t="n">
+        <v>421.05</v>
+      </c>
+      <c r="AL3" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="AM3" s="5" t="n">
+        <v>369.59</v>
+      </c>
+      <c r="AN3" s="5" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="AO3" s="5" t="n">
+        <v>-2.07</v>
+      </c>
+      <c r="AP3" s="5" t="n">
         <v>0</v>
-      </c>
-      <c r="N3" s="5" t="n">
-        <v>86.5</v>
-      </c>
-      <c r="O3" s="5" t="inlineStr">
-        <is>
-          <t>STRONG</t>
-        </is>
-      </c>
-      <c r="P3" s="5" t="inlineStr">
-        <is>
-          <t>🟢</t>
-        </is>
-      </c>
-      <c r="Q3" s="5" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="R3" s="5" t="n">
-        <v>-0.8</v>
-      </c>
-      <c r="S3" s="5" t="inlineStr">
-        <is>
-          <t>crude +19.8% (rising) → +1.0pts · 5 insider Form 4 filings last 90d → +1.0pts (note: buy/sell parse pending)</t>
-        </is>
-      </c>
-      <c r="T3" s="5" t="inlineStr">
-        <is>
-          <t>🟢 BUY (Δ-3.0%) · Rank → 2→2 · Conf 54% · band STRONG · 14d left · → HOLD</t>
-        </is>
-      </c>
-      <c r="U3" s="5" t="inlineStr"/>
-      <c r="V3" s="5" t="n">
-        <v>53.6</v>
-      </c>
-      <c r="W3" s="5" t="inlineStr">
-        <is>
-          <t>Calibrated</t>
-        </is>
-      </c>
-      <c r="X3" s="5" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="Y3" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="Z3" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="AA3" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="AB3" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="AC3" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="AD3" s="5" t="n">
-        <v>358.56</v>
-      </c>
-      <c r="AE3" s="5" t="n">
-        <v>366.13</v>
-      </c>
-      <c r="AF3" s="5" t="n">
-        <v>362.47</v>
-      </c>
-      <c r="AG3" s="5" t="n">
-        <v>369.79</v>
-      </c>
-      <c r="AH3" s="5" t="n">
-        <v>347.82</v>
-      </c>
-      <c r="AI3" s="5" t="n">
-        <v>-5</v>
-      </c>
-      <c r="AJ3" s="5" t="n">
-        <v>395.42</v>
-      </c>
-      <c r="AK3" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="AL3" s="5" t="n">
-        <v>421.05</v>
-      </c>
-      <c r="AM3" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="AN3" s="5" t="n">
-        <v>369.59</v>
-      </c>
-      <c r="AO3" s="5" t="n">
-        <v>-0.28</v>
-      </c>
-      <c r="AP3" s="5" t="n">
-        <v>-2.07</v>
       </c>
       <c r="AQ3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AR3" s="5" t="n">
+      <c r="AR3" s="5" t="inlineStr">
+        <is>
+          <t>Momentum · Trend · Quality</t>
+        </is>
+      </c>
+      <c r="AS3" s="5" t="inlineStr"/>
+      <c r="AT3" s="5" t="inlineStr"/>
+      <c r="AU3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AS3" s="5" t="inlineStr">
-        <is>
-          <t>Momentum · Trend · Quality</t>
-        </is>
-      </c>
-      <c r="AT3" s="5" t="inlineStr"/>
-      <c r="AU3" s="5" t="inlineStr"/>
-      <c r="AV3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW3" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-07 09:51</t>
+      <c r="AV3" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:01</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1100,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>R1_NEW</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1134,134 +1118,129 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="H4" s="3" t="inlineStr"/>
       <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="n">
+      <c r="J4" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="K4" s="3" t="inlineStr"/>
       <c r="L4" s="3" t="inlineStr"/>
-      <c r="M4" s="3" t="inlineStr"/>
-      <c r="N4" s="3" t="n">
+      <c r="M4" s="3" t="n">
         <v>86.5</v>
       </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>STRONG</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
           <t>🟢</t>
         </is>
       </c>
+      <c r="P4" s="3" t="n">
+        <v>52.9</v>
+      </c>
       <c r="Q4" s="3" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="R4" s="3" t="n">
         <v>-0.8</v>
       </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>crude +19.8% (rising) → +1.0pts · 5 insider Form 4 filings last 90d → +1.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>crude +19.8% (rising) → +1.0pts · 5 insider Form 4 filings last 90d → +1.0pts (note: buy/sell parse pending)</t>
-        </is>
-      </c>
-      <c r="T4" s="3" t="inlineStr">
-        <is>
           <t>🟢 BUY (Δ-2.0%) · Rank #1 · Conf 54% · momentum → · band STRONG · 91d left · → BUY</t>
         </is>
       </c>
-      <c r="U4" s="3" t="inlineStr"/>
-      <c r="V4" s="3" t="n">
+      <c r="T4" s="3" t="inlineStr"/>
+      <c r="U4" s="3" t="n">
         <v>53.6</v>
       </c>
-      <c r="W4" s="3" t="inlineStr">
+      <c r="V4" s="3" t="inlineStr">
         <is>
           <t>Calibrated</t>
         </is>
       </c>
-      <c r="X4" s="3" t="n">
+      <c r="W4" s="3" t="n">
         <v>64.3</v>
       </c>
-      <c r="Y4" s="3" t="inlineStr"/>
+      <c r="X4" s="3" t="inlineStr"/>
+      <c r="Y4" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="Z4" s="3" t="n">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="AA4" s="3" t="n">
-        <v>90</v>
-      </c>
-      <c r="AB4" s="3" t="n">
         <v>91</v>
       </c>
-      <c r="AC4" s="3" t="inlineStr">
+      <c r="AB4" s="3" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
+      <c r="AC4" s="3" t="n">
+        <v>358.56</v>
+      </c>
       <c r="AD4" s="3" t="n">
-        <v>358.56</v>
+        <v>366.13</v>
       </c>
       <c r="AE4" s="3" t="n">
-        <v>366.13</v>
+        <v>351.39</v>
       </c>
       <c r="AF4" s="3" t="n">
-        <v>351.39</v>
+        <v>365.73</v>
       </c>
       <c r="AG4" s="3" t="n">
-        <v>365.73</v>
+        <v>340.632</v>
       </c>
       <c r="AH4" s="3" t="n">
-        <v>340.632</v>
+        <v>-6.96</v>
       </c>
       <c r="AI4" s="3" t="n">
-        <v>-6.96</v>
+        <v>387.2448000000001</v>
       </c>
       <c r="AJ4" s="3" t="n">
-        <v>387.2448000000001</v>
+        <v>5.77</v>
       </c>
       <c r="AK4" s="3" t="n">
-        <v>5.77</v>
+        <v>414.3519360000001</v>
       </c>
       <c r="AL4" s="3" t="n">
-        <v>414.3519360000001</v>
+        <v>13.17</v>
       </c>
       <c r="AM4" s="3" t="n">
-        <v>13.17</v>
+        <v>369.59</v>
       </c>
       <c r="AN4" s="3" t="n">
-        <v>369.59</v>
+        <v>-0.28</v>
       </c>
       <c r="AO4" s="3" t="n">
-        <v>-0.28</v>
+        <v>-2.07</v>
       </c>
       <c r="AP4" s="3" t="n">
-        <v>-2.07</v>
+        <v>0</v>
       </c>
       <c r="AQ4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AR4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS4" s="3" t="inlineStr"/>
-      <c r="AT4" s="3" t="inlineStr">
+      <c r="AR4" s="3" t="inlineStr"/>
+      <c r="AS4" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AT4" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AU4" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AV4" s="3" t="n">
         <v>5.77</v>
       </c>
-      <c r="AW4" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-07 09:51</t>
+      <c r="AV4" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:01</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1262,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>R1_NEW</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1301,134 +1280,129 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="n">
+      <c r="J5" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="K5" s="3" t="inlineStr"/>
       <c r="L5" s="3" t="inlineStr"/>
-      <c r="M5" s="3" t="inlineStr"/>
-      <c r="N5" s="3" t="n">
+      <c r="M5" s="3" t="n">
         <v>79.3</v>
       </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="P5" s="3" t="inlineStr">
-        <is>
           <t>🟢</t>
         </is>
       </c>
+      <c r="P5" s="3" t="n">
+        <v>56.1</v>
+      </c>
       <c r="Q5" s="3" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="R5" s="3" t="n">
         <v>-0.8</v>
       </c>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>crude +19.8% (rising) → +1.0pts · 12 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>crude +19.8% (rising) → +1.0pts · 12 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
-        </is>
-      </c>
-      <c r="T5" s="3" t="inlineStr">
-        <is>
           <t>🟢 BUY (Δ-1.0%) · Rank #2 · Conf 57% · momentum → · band HOLD · 91d left · → BUY</t>
         </is>
       </c>
-      <c r="U5" s="3" t="inlineStr"/>
-      <c r="V5" s="3" t="n">
+      <c r="T5" s="3" t="inlineStr"/>
+      <c r="U5" s="3" t="n">
         <v>56.8</v>
       </c>
-      <c r="W5" s="3" t="inlineStr">
+      <c r="V5" s="3" t="inlineStr">
         <is>
           <t>Calibrated</t>
         </is>
       </c>
-      <c r="X5" s="3" t="n">
+      <c r="W5" s="3" t="n">
         <v>58.8</v>
       </c>
-      <c r="Y5" s="3" t="inlineStr"/>
+      <c r="X5" s="3" t="inlineStr"/>
+      <c r="Y5" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="Z5" s="3" t="n">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="AA5" s="3" t="n">
-        <v>90</v>
-      </c>
-      <c r="AB5" s="3" t="n">
         <v>91</v>
       </c>
-      <c r="AC5" s="3" t="inlineStr">
+      <c r="AB5" s="3" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
+      <c r="AC5" s="3" t="n">
+        <v>368.98</v>
+      </c>
       <c r="AD5" s="3" t="n">
-        <v>368.98</v>
+        <v>374.36</v>
       </c>
       <c r="AE5" s="3" t="n">
-        <v>374.36</v>
+        <v>365.29</v>
       </c>
       <c r="AF5" s="3" t="n">
-        <v>365.29</v>
+        <v>372.67</v>
       </c>
       <c r="AG5" s="3" t="n">
-        <v>372.67</v>
+        <v>350.531</v>
       </c>
       <c r="AH5" s="3" t="n">
-        <v>350.531</v>
+        <v>-6.37</v>
       </c>
       <c r="AI5" s="3" t="n">
-        <v>-6.37</v>
+        <v>413.26</v>
       </c>
       <c r="AJ5" s="3" t="n">
-        <v>413.26</v>
+        <v>10.39</v>
       </c>
       <c r="AK5" s="3" t="n">
-        <v>10.39</v>
+        <v>442.1882</v>
       </c>
       <c r="AL5" s="3" t="n">
-        <v>442.1882</v>
+        <v>18.12</v>
       </c>
       <c r="AM5" s="3" t="n">
-        <v>18.12</v>
+        <v>377.15</v>
       </c>
       <c r="AN5" s="3" t="n">
-        <v>377.15</v>
+        <v>1.41</v>
       </c>
       <c r="AO5" s="3" t="n">
-        <v>1.41</v>
+        <v>-1.44</v>
       </c>
       <c r="AP5" s="3" t="n">
-        <v>-1.44</v>
+        <v>0</v>
       </c>
       <c r="AQ5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AR5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS5" s="3" t="inlineStr"/>
-      <c r="AT5" s="3" t="inlineStr">
+      <c r="AR5" s="3" t="inlineStr"/>
+      <c r="AS5" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AT5" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AU5" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AV5" s="3" t="n">
         <v>10.39</v>
       </c>
-      <c r="AW5" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-07 09:51</t>
+      <c r="AV5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:01</t>
         </is>
       </c>
     </row>
@@ -1450,7 +1424,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>R1_NEW</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1468,134 +1442,129 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr"/>
-      <c r="K6" s="3" t="n">
+      <c r="J6" s="3" t="n">
         <v>3</v>
       </c>
+      <c r="K6" s="3" t="inlineStr"/>
       <c r="L6" s="3" t="inlineStr"/>
-      <c r="M6" s="3" t="inlineStr"/>
-      <c r="N6" s="3" t="n">
+      <c r="M6" s="3" t="n">
         <v>67.5</v>
       </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="P6" s="3" t="inlineStr">
-        <is>
           <t>🟢</t>
         </is>
       </c>
+      <c r="P6" s="3" t="n">
+        <v>46.6</v>
+      </c>
       <c r="Q6" s="3" t="n">
-        <v>46.6</v>
-      </c>
-      <c r="R6" s="3" t="n">
         <v>-0.8</v>
       </c>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>crude +19.8% (rising) → +1.0pts · 21 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>crude +19.8% (rising) → +1.0pts · 21 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
-        </is>
-      </c>
-      <c r="T6" s="3" t="inlineStr">
-        <is>
           <t>🟢 BUY (Δ-2.0%) · Rank #3 · Conf 47% · momentum → · band HOLD · 91d left · → BUY</t>
         </is>
       </c>
-      <c r="U6" s="3" t="inlineStr"/>
-      <c r="V6" s="3" t="n">
+      <c r="T6" s="3" t="inlineStr"/>
+      <c r="U6" s="3" t="n">
         <v>47.3</v>
       </c>
-      <c r="W6" s="3" t="inlineStr">
+      <c r="V6" s="3" t="inlineStr">
         <is>
           <t>Calibrated</t>
         </is>
       </c>
-      <c r="X6" s="3" t="n">
+      <c r="W6" s="3" t="n">
         <v>55.7</v>
       </c>
-      <c r="Y6" s="3" t="inlineStr"/>
+      <c r="X6" s="3" t="inlineStr"/>
+      <c r="Y6" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="Z6" s="3" t="n">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="AA6" s="3" t="n">
-        <v>90</v>
-      </c>
-      <c r="AB6" s="3" t="n">
         <v>91</v>
       </c>
-      <c r="AC6" s="3" t="inlineStr">
+      <c r="AB6" s="3" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
+      <c r="AC6" s="3" t="n">
+        <v>202.81</v>
+      </c>
       <c r="AD6" s="3" t="n">
-        <v>202.81</v>
+        <v>200.75</v>
       </c>
       <c r="AE6" s="3" t="n">
-        <v>200.75</v>
+        <v>198.75</v>
       </c>
       <c r="AF6" s="3" t="n">
-        <v>198.75</v>
+        <v>206.87</v>
       </c>
       <c r="AG6" s="3" t="n">
-        <v>206.87</v>
+        <v>192.6695</v>
       </c>
       <c r="AH6" s="3" t="n">
-        <v>192.6695</v>
+        <v>-4.03</v>
       </c>
       <c r="AI6" s="3" t="n">
-        <v>-4.03</v>
+        <v>219.0348</v>
       </c>
       <c r="AJ6" s="3" t="n">
-        <v>219.0348</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="AK6" s="3" t="n">
-        <v>9.109999999999999</v>
+        <v>234.367236</v>
       </c>
       <c r="AL6" s="3" t="n">
-        <v>234.367236</v>
+        <v>16.75</v>
       </c>
       <c r="AM6" s="3" t="n">
-        <v>16.75</v>
+        <v>211.94</v>
       </c>
       <c r="AN6" s="3" t="n">
-        <v>211.94</v>
+        <v>3.43</v>
       </c>
       <c r="AO6" s="3" t="n">
-        <v>3.43</v>
+        <v>1.03</v>
       </c>
       <c r="AP6" s="3" t="n">
-        <v>1.03</v>
+        <v>0</v>
       </c>
       <c r="AQ6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AR6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS6" s="3" t="inlineStr"/>
-      <c r="AT6" s="3" t="inlineStr">
+      <c r="AR6" s="3" t="inlineStr"/>
+      <c r="AS6" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AT6" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AU6" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AV6" s="3" t="n">
         <v>9.109999999999999</v>
       </c>
-      <c r="AW6" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-07 09:51</t>
+      <c r="AV6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:01</t>
         </is>
       </c>
     </row>
@@ -1617,7 +1586,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>R1_NEW</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1635,138 +1604,133 @@
           <t>BUY</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="n">
+      <c r="J7" s="3" t="n">
         <v>4</v>
       </c>
+      <c r="K7" s="3" t="inlineStr"/>
       <c r="L7" s="3" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr"/>
-      <c r="N7" s="3" t="n">
+      <c r="M7" s="3" t="n">
         <v>79.5</v>
       </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="P7" s="3" t="inlineStr">
-        <is>
           <t>🟢</t>
         </is>
       </c>
+      <c r="P7" s="3" t="n">
+        <v>52.9</v>
+      </c>
       <c r="Q7" s="3" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="R7" s="3" t="n">
         <v>-0.8</v>
       </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>crude +19.8% (rising) → +1.0pts · 33 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>crude +19.8% (rising) → +1.0pts · 33 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+          <t>🟢 BUY (Δ-2.0%) · Rank #4 · Conf 54% · momentum → · band HOLD · 91d left · → BUY</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>🟢 BUY (Δ-2.0%) · Rank #4 · Conf 54% · momentum → · band HOLD · 91d left · → BUY</t>
-        </is>
-      </c>
-      <c r="U7" s="3" t="inlineStr">
-        <is>
           <t>CRITICAL·DEEP_LOSS·-15.3% ≤ -8% · EXIT URGENT</t>
         </is>
       </c>
-      <c r="V7" s="3" t="n">
+      <c r="U7" s="3" t="n">
         <v>53.6</v>
       </c>
-      <c r="W7" s="3" t="inlineStr">
+      <c r="V7" s="3" t="inlineStr">
         <is>
           <t>Calibrated</t>
         </is>
       </c>
-      <c r="X7" s="3" t="n">
+      <c r="W7" s="3" t="n">
         <v>51.8</v>
       </c>
-      <c r="Y7" s="3" t="inlineStr"/>
+      <c r="X7" s="3" t="inlineStr"/>
+      <c r="Y7" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="Z7" s="3" t="n">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="AA7" s="3" t="n">
-        <v>90</v>
-      </c>
-      <c r="AB7" s="3" t="n">
         <v>91</v>
       </c>
-      <c r="AC7" s="3" t="inlineStr">
+      <c r="AB7" s="3" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
+      <c r="AC7" s="3" t="n">
+        <v>393.82</v>
+      </c>
       <c r="AD7" s="3" t="n">
-        <v>393.82</v>
+        <v>464.72</v>
       </c>
       <c r="AE7" s="3" t="n">
-        <v>464.72</v>
+        <v>385.94</v>
       </c>
       <c r="AF7" s="3" t="n">
-        <v>385.94</v>
+        <v>401.7</v>
       </c>
       <c r="AG7" s="3" t="n">
-        <v>401.7</v>
+        <v>374.129</v>
       </c>
       <c r="AH7" s="3" t="n">
-        <v>374.129</v>
+        <v>-19.49</v>
       </c>
       <c r="AI7" s="3" t="n">
-        <v>-19.49</v>
+        <v>425.3256</v>
       </c>
       <c r="AJ7" s="3" t="n">
-        <v>425.3256</v>
+        <v>-8.48</v>
       </c>
       <c r="AK7" s="3" t="n">
-        <v>-8.48</v>
+        <v>455.098392</v>
       </c>
       <c r="AL7" s="3" t="n">
-        <v>455.098392</v>
+        <v>-2.07</v>
       </c>
       <c r="AM7" s="3" t="n">
-        <v>-2.07</v>
+        <v>492.81</v>
       </c>
       <c r="AN7" s="3" t="n">
-        <v>492.81</v>
+        <v>-1.09</v>
       </c>
       <c r="AO7" s="3" t="n">
-        <v>-1.09</v>
+        <v>-15.26</v>
       </c>
       <c r="AP7" s="3" t="n">
-        <v>-15.26</v>
+        <v>0</v>
       </c>
       <c r="AQ7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AR7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS7" s="3" t="inlineStr"/>
-      <c r="AT7" s="3" t="inlineStr">
+      <c r="AR7" s="3" t="inlineStr"/>
+      <c r="AS7" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AT7" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AU7" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AV7" s="3" t="n">
         <v>-8.48</v>
       </c>
-      <c r="AW7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-07 09:51</t>
+      <c r="AV7" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:01</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1752,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>R1_NEW</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -1806,138 +1770,133 @@
           <t>HOLD</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="H8" s="5" t="inlineStr"/>
       <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="5" t="inlineStr"/>
-      <c r="K8" s="5" t="n">
+      <c r="J8" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="K8" s="5" t="inlineStr"/>
       <c r="L8" s="5" t="inlineStr"/>
-      <c r="M8" s="5" t="inlineStr"/>
-      <c r="N8" s="5" t="n">
+      <c r="M8" s="5" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>STRONG</t>
-        </is>
-      </c>
-      <c r="P8" s="5" t="inlineStr">
-        <is>
           <t>🟢</t>
         </is>
       </c>
+      <c r="P8" s="5" t="n">
+        <v>49.7</v>
+      </c>
       <c r="Q8" s="5" t="n">
-        <v>49.7</v>
-      </c>
-      <c r="R8" s="5" t="n">
         <v>-0.8</v>
       </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>crude +19.8% (rising) → +1.0pts · 11 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>crude +19.8% (rising) → +1.0pts · 11 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+          <t>🟢 BUY (Δ-2.0%) · Rank #5 · Conf 50% · momentum → · band STRONG · 91d left · → HOLD</t>
         </is>
       </c>
       <c r="T8" s="5" t="inlineStr">
         <is>
-          <t>🟢 BUY (Δ-2.0%) · Rank #5 · Conf 50% · momentum → · band STRONG · 91d left · → HOLD</t>
-        </is>
-      </c>
-      <c r="U8" s="5" t="inlineStr">
-        <is>
           <t>WARNING·STOP_LOSS_HIT·-6.9% ≤ -5% · exit</t>
         </is>
       </c>
-      <c r="V8" s="5" t="n">
+      <c r="U8" s="5" t="n">
         <v>50.5</v>
       </c>
-      <c r="W8" s="5" t="inlineStr">
+      <c r="V8" s="5" t="inlineStr">
         <is>
           <t>Calibrated</t>
         </is>
       </c>
-      <c r="X8" s="5" t="n">
+      <c r="W8" s="5" t="n">
         <v>46.7</v>
       </c>
-      <c r="Y8" s="5" t="inlineStr"/>
+      <c r="X8" s="5" t="inlineStr"/>
+      <c r="Y8" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="Z8" s="5" t="n">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="AA8" s="5" t="n">
-        <v>90</v>
-      </c>
-      <c r="AB8" s="5" t="n">
         <v>91</v>
       </c>
-      <c r="AC8" s="5" t="inlineStr">
+      <c r="AB8" s="5" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
+      <c r="AC8" s="5" t="n">
+        <v>81.56</v>
+      </c>
       <c r="AD8" s="5" t="n">
-        <v>81.56</v>
+        <v>87.59</v>
       </c>
       <c r="AE8" s="5" t="n">
-        <v>87.59</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="AF8" s="5" t="n">
-        <v>79.93000000000001</v>
+        <v>83.19</v>
       </c>
       <c r="AG8" s="5" t="n">
-        <v>83.19</v>
+        <v>77.482</v>
       </c>
       <c r="AH8" s="5" t="n">
-        <v>77.482</v>
+        <v>-11.54</v>
       </c>
       <c r="AI8" s="5" t="n">
-        <v>-11.54</v>
+        <v>88.0848</v>
       </c>
       <c r="AJ8" s="5" t="n">
-        <v>88.0848</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>94.250736</v>
       </c>
       <c r="AL8" s="5" t="n">
-        <v>94.250736</v>
+        <v>7.6</v>
       </c>
       <c r="AM8" s="5" t="n">
-        <v>7.6</v>
+        <v>86.56</v>
       </c>
       <c r="AN8" s="5" t="n">
-        <v>86.56</v>
+        <v>0.31</v>
       </c>
       <c r="AO8" s="5" t="n">
-        <v>0.31</v>
+        <v>-6.88</v>
       </c>
       <c r="AP8" s="5" t="n">
-        <v>-6.88</v>
+        <v>0</v>
       </c>
       <c r="AQ8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AR8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS8" s="5" t="inlineStr"/>
-      <c r="AT8" s="5" t="inlineStr">
+      <c r="AR8" s="5" t="inlineStr"/>
+      <c r="AS8" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AT8" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="AU8" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="AV8" s="5" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="AW8" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-07 09:51</t>
+      <c r="AV8" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:01</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1918,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>R1_NEW</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -1977,138 +1936,133 @@
           <t>HOLD</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="H9" s="5" t="inlineStr"/>
       <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr"/>
-      <c r="K9" s="5" t="n">
+      <c r="J9" s="5" t="n">
         <v>6</v>
       </c>
+      <c r="K9" s="5" t="inlineStr"/>
       <c r="L9" s="5" t="inlineStr"/>
-      <c r="M9" s="5" t="inlineStr"/>
-      <c r="N9" s="5" t="n">
+      <c r="M9" s="5" t="n">
         <v>76</v>
       </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="P9" s="5" t="inlineStr">
-        <is>
           <t>🟢</t>
         </is>
       </c>
+      <c r="P9" s="5" t="n">
+        <v>49.7</v>
+      </c>
       <c r="Q9" s="5" t="n">
-        <v>49.7</v>
-      </c>
-      <c r="R9" s="5" t="n">
         <v>-0.8</v>
       </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>crude +19.8% (rising) → +1.0pts · 48 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
       <c r="S9" s="5" t="inlineStr">
         <is>
-          <t>crude +19.8% (rising) → +1.0pts · 48 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+          <t>🟢 BUY (Δ-2.0%) · Rank #6 · Conf 50% · momentum → · band HOLD · 91d left · → HOLD</t>
         </is>
       </c>
       <c r="T9" s="5" t="inlineStr">
         <is>
-          <t>🟢 BUY (Δ-2.0%) · Rank #6 · Conf 50% · momentum → · band HOLD · 91d left · → HOLD</t>
-        </is>
-      </c>
-      <c r="U9" s="5" t="inlineStr">
-        <is>
           <t>WARNING·STOP_LOSS_HIT·-7.4% ≤ -5% · exit</t>
         </is>
       </c>
-      <c r="V9" s="5" t="n">
+      <c r="U9" s="5" t="n">
         <v>50.5</v>
       </c>
-      <c r="W9" s="5" t="inlineStr">
+      <c r="V9" s="5" t="inlineStr">
         <is>
           <t>Calibrated</t>
         </is>
       </c>
-      <c r="X9" s="5" t="n">
+      <c r="W9" s="5" t="n">
         <v>46.5</v>
       </c>
-      <c r="Y9" s="5" t="inlineStr"/>
+      <c r="X9" s="5" t="inlineStr"/>
+      <c r="Y9" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="Z9" s="5" t="n">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="AA9" s="5" t="n">
-        <v>90</v>
-      </c>
-      <c r="AB9" s="5" t="n">
         <v>91</v>
       </c>
-      <c r="AC9" s="5" t="inlineStr">
+      <c r="AB9" s="5" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
+      <c r="AC9" s="5" t="n">
+        <v>225.02</v>
+      </c>
       <c r="AD9" s="5" t="n">
-        <v>225.02</v>
+        <v>243.05</v>
       </c>
       <c r="AE9" s="5" t="n">
-        <v>243.05</v>
+        <v>220.52</v>
       </c>
       <c r="AF9" s="5" t="n">
-        <v>220.52</v>
+        <v>229.52</v>
       </c>
       <c r="AG9" s="5" t="n">
-        <v>229.52</v>
+        <v>213.769</v>
       </c>
       <c r="AH9" s="5" t="n">
-        <v>213.769</v>
+        <v>-12.05</v>
       </c>
       <c r="AI9" s="5" t="n">
-        <v>-12.05</v>
+        <v>243.0216</v>
       </c>
       <c r="AJ9" s="5" t="n">
-        <v>243.0216</v>
+        <v>-0.01</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>-0.01</v>
+        <v>260.0331120000001</v>
       </c>
       <c r="AL9" s="5" t="n">
-        <v>260.0331120000001</v>
+        <v>6.99</v>
       </c>
       <c r="AM9" s="5" t="n">
-        <v>6.99</v>
+        <v>248.79</v>
       </c>
       <c r="AN9" s="5" t="n">
-        <v>248.79</v>
+        <v>-0.27</v>
       </c>
       <c r="AO9" s="5" t="n">
-        <v>-0.27</v>
+        <v>-7.42</v>
       </c>
       <c r="AP9" s="5" t="n">
-        <v>-7.42</v>
+        <v>0</v>
       </c>
       <c r="AQ9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AR9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS9" s="5" t="inlineStr"/>
-      <c r="AT9" s="5" t="inlineStr">
+      <c r="AR9" s="5" t="inlineStr"/>
+      <c r="AS9" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AT9" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="AU9" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="AV9" s="5" t="n">
         <v>-0.01</v>
       </c>
-      <c r="AW9" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-07 09:51</t>
+      <c r="AV9" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:01</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2084,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>R1_NEW</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -2148,134 +2102,129 @@
           <t>HOLD</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="H10" s="5" t="inlineStr"/>
       <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr"/>
-      <c r="K10" s="5" t="n">
+      <c r="J10" s="5" t="n">
         <v>7</v>
       </c>
+      <c r="K10" s="5" t="inlineStr"/>
       <c r="L10" s="5" t="inlineStr"/>
-      <c r="M10" s="5" t="inlineStr"/>
-      <c r="N10" s="5" t="n">
+      <c r="M10" s="5" t="n">
         <v>83.5</v>
       </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
-          <t>STRONG</t>
-        </is>
-      </c>
-      <c r="P10" s="5" t="inlineStr">
-        <is>
           <t>🟢</t>
         </is>
       </c>
+      <c r="P10" s="5" t="n">
+        <v>49.7</v>
+      </c>
       <c r="Q10" s="5" t="n">
-        <v>49.7</v>
-      </c>
-      <c r="R10" s="5" t="n">
         <v>-0.8</v>
       </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>crude +19.8% (rising) → +1.0pts · 5 insider Form 4 filings last 90d → +1.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>crude +19.8% (rising) → +1.0pts · 5 insider Form 4 filings last 90d → +1.0pts (note: buy/sell parse pending)</t>
-        </is>
-      </c>
-      <c r="T10" s="5" t="inlineStr">
-        <is>
           <t>🟢 BUY (Δ-2.0%) · Rank #7 · Conf 50% · momentum → · band STRONG · 91d left · → HOLD</t>
         </is>
       </c>
-      <c r="U10" s="5" t="inlineStr"/>
-      <c r="V10" s="5" t="n">
+      <c r="T10" s="5" t="inlineStr"/>
+      <c r="U10" s="5" t="n">
         <v>50.5</v>
       </c>
-      <c r="W10" s="5" t="inlineStr">
+      <c r="V10" s="5" t="inlineStr">
         <is>
           <t>Calibrated</t>
         </is>
       </c>
-      <c r="X10" s="5" t="n">
+      <c r="W10" s="5" t="n">
         <v>45.8</v>
       </c>
-      <c r="Y10" s="5" t="inlineStr"/>
+      <c r="X10" s="5" t="inlineStr"/>
+      <c r="Y10" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="Z10" s="5" t="n">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="AA10" s="5" t="n">
-        <v>90</v>
-      </c>
-      <c r="AB10" s="5" t="n">
         <v>91</v>
       </c>
-      <c r="AC10" s="5" t="inlineStr">
+      <c r="AB10" s="5" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
+      <c r="AC10" s="5" t="n">
+        <v>333.74</v>
+      </c>
       <c r="AD10" s="5" t="n">
-        <v>333.74</v>
+        <v>308.91</v>
       </c>
       <c r="AE10" s="5" t="n">
-        <v>308.91</v>
+        <v>327.07</v>
       </c>
       <c r="AF10" s="5" t="n">
-        <v>327.07</v>
+        <v>340.41</v>
       </c>
       <c r="AG10" s="5" t="n">
-        <v>340.41</v>
+        <v>317.053</v>
       </c>
       <c r="AH10" s="5" t="n">
-        <v>317.053</v>
+        <v>2.64</v>
       </c>
       <c r="AI10" s="5" t="n">
-        <v>2.64</v>
+        <v>360.4392</v>
       </c>
       <c r="AJ10" s="5" t="n">
-        <v>360.4392</v>
+        <v>16.68</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>16.68</v>
+        <v>385.669944</v>
       </c>
       <c r="AL10" s="5" t="n">
-        <v>385.669944</v>
+        <v>24.85</v>
       </c>
       <c r="AM10" s="5" t="n">
-        <v>24.85</v>
+        <v>309.38</v>
       </c>
       <c r="AN10" s="5" t="n">
-        <v>309.38</v>
+        <v>0.52</v>
       </c>
       <c r="AO10" s="5" t="n">
-        <v>0.52</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="AP10" s="5" t="n">
-        <v>8.039999999999999</v>
+        <v>0</v>
       </c>
       <c r="AQ10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AR10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS10" s="5" t="inlineStr"/>
-      <c r="AT10" s="5" t="inlineStr">
+      <c r="AR10" s="5" t="inlineStr"/>
+      <c r="AS10" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AT10" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="AU10" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="AV10" s="5" t="n">
         <v>16.68</v>
       </c>
-      <c r="AW10" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-07 09:51</t>
+      <c r="AV10" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:01</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2246,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>R1_NEW</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -2315,134 +2264,129 @@
           <t>HOLD</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="H11" s="5" t="inlineStr"/>
       <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr"/>
-      <c r="K11" s="5" t="n">
+      <c r="J11" s="5" t="n">
         <v>8</v>
       </c>
+      <c r="K11" s="5" t="inlineStr"/>
       <c r="L11" s="5" t="inlineStr"/>
-      <c r="M11" s="5" t="inlineStr"/>
-      <c r="N11" s="5" t="n">
+      <c r="M11" s="5" t="n">
         <v>78.40000000000001</v>
       </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="P11" s="5" t="inlineStr">
-        <is>
           <t>🟢</t>
         </is>
       </c>
+      <c r="P11" s="5" t="n">
+        <v>48.9</v>
+      </c>
       <c r="Q11" s="5" t="n">
-        <v>48.9</v>
-      </c>
-      <c r="R11" s="5" t="n">
         <v>-0.8</v>
       </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>crude +19.8% (rising) → +1.0pts · 18 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
       <c r="S11" s="5" t="inlineStr">
         <is>
-          <t>crude +19.8% (rising) → +1.0pts · 18 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
-        </is>
-      </c>
-      <c r="T11" s="5" t="inlineStr">
-        <is>
           <t>🟢 BUY (Δ-2.0%) · Rank #8 · Conf 50% · momentum → · band HOLD · 91d left · → HOLD</t>
         </is>
       </c>
-      <c r="U11" s="5" t="inlineStr"/>
-      <c r="V11" s="5" t="n">
+      <c r="T11" s="5" t="inlineStr"/>
+      <c r="U11" s="5" t="n">
         <v>49.7</v>
       </c>
-      <c r="W11" s="5" t="inlineStr">
+      <c r="V11" s="5" t="inlineStr">
         <is>
           <t>Calibrated</t>
         </is>
       </c>
-      <c r="X11" s="5" t="n">
+      <c r="W11" s="5" t="n">
         <v>37.6</v>
       </c>
-      <c r="Y11" s="5" t="inlineStr"/>
+      <c r="X11" s="5" t="inlineStr"/>
+      <c r="Y11" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="Z11" s="5" t="n">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="AA11" s="5" t="n">
-        <v>90</v>
-      </c>
-      <c r="AB11" s="5" t="n">
         <v>91</v>
       </c>
-      <c r="AC11" s="5" t="inlineStr">
+      <c r="AB11" s="5" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
+      <c r="AC11" s="5" t="n">
+        <v>341.1</v>
+      </c>
       <c r="AD11" s="5" t="n">
-        <v>341.1</v>
+        <v>351.79</v>
       </c>
       <c r="AE11" s="5" t="n">
-        <v>351.79</v>
+        <v>334.28</v>
       </c>
       <c r="AF11" s="5" t="n">
-        <v>334.28</v>
+        <v>347.92</v>
       </c>
       <c r="AG11" s="5" t="n">
-        <v>347.92</v>
+        <v>324.045</v>
       </c>
       <c r="AH11" s="5" t="n">
-        <v>324.045</v>
+        <v>-7.89</v>
       </c>
       <c r="AI11" s="5" t="n">
-        <v>-7.89</v>
+        <v>368.388</v>
       </c>
       <c r="AJ11" s="5" t="n">
-        <v>368.388</v>
+        <v>4.72</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>4.72</v>
+        <v>394.1751600000001</v>
       </c>
       <c r="AL11" s="5" t="n">
-        <v>394.1751600000001</v>
+        <v>12.05</v>
       </c>
       <c r="AM11" s="5" t="n">
-        <v>12.05</v>
+        <v>357.52</v>
       </c>
       <c r="AN11" s="5" t="n">
-        <v>357.52</v>
+        <v>0.48</v>
       </c>
       <c r="AO11" s="5" t="n">
-        <v>0.48</v>
+        <v>-3.04</v>
       </c>
       <c r="AP11" s="5" t="n">
-        <v>-3.04</v>
+        <v>0</v>
       </c>
       <c r="AQ11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AR11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS11" s="5" t="inlineStr"/>
-      <c r="AT11" s="5" t="inlineStr">
+      <c r="AR11" s="5" t="inlineStr"/>
+      <c r="AS11" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AT11" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="AU11" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="AV11" s="5" t="n">
         <v>4.72</v>
       </c>
-      <c r="AW11" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-07 09:51</t>
+      <c r="AV11" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:01</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2408,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>R1_NEW</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -2482,134 +2426,129 @@
           <t>HOLD</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="H12" s="5" t="inlineStr"/>
       <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="5" t="inlineStr"/>
-      <c r="K12" s="5" t="n">
+      <c r="J12" s="5" t="n">
         <v>9</v>
       </c>
+      <c r="K12" s="5" t="inlineStr"/>
       <c r="L12" s="5" t="inlineStr"/>
-      <c r="M12" s="5" t="inlineStr"/>
-      <c r="N12" s="5" t="n">
+      <c r="M12" s="5" t="n">
         <v>66.3</v>
       </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="P12" s="5" t="inlineStr">
-        <is>
           <t>🟢</t>
         </is>
       </c>
+      <c r="P12" s="5" t="n">
+        <v>50.2</v>
+      </c>
       <c r="Q12" s="5" t="n">
-        <v>50.2</v>
-      </c>
-      <c r="R12" s="5" t="n">
         <v>-0.8</v>
       </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>crude +19.8% (rising) → +1.0pts · 9 insider Form 4 filings last 90d → +1.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>crude +19.8% (rising) → +1.0pts · 9 insider Form 4 filings last 90d → +1.0pts (note: buy/sell parse pending)</t>
-        </is>
-      </c>
-      <c r="T12" s="5" t="inlineStr">
-        <is>
           <t>🟢 BUY (Δ-2.0%) · Rank #9 · Conf 51% · momentum → · band HOLD · 91d left · → HOLD</t>
         </is>
       </c>
-      <c r="U12" s="5" t="inlineStr"/>
-      <c r="V12" s="5" t="n">
+      <c r="T12" s="5" t="inlineStr"/>
+      <c r="U12" s="5" t="n">
         <v>51</v>
       </c>
-      <c r="W12" s="5" t="inlineStr">
+      <c r="V12" s="5" t="inlineStr">
         <is>
           <t>Calibrated</t>
         </is>
       </c>
-      <c r="X12" s="5" t="n">
+      <c r="W12" s="5" t="n">
         <v>36.5</v>
       </c>
-      <c r="Y12" s="5" t="inlineStr"/>
+      <c r="X12" s="5" t="inlineStr"/>
+      <c r="Y12" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="Z12" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="AA12" s="5" t="n">
+        <v>91</v>
+      </c>
+      <c r="AB12" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="AC12" s="5" t="n">
+        <v>1065.22</v>
+      </c>
+      <c r="AD12" s="5" t="n">
+        <v>1018.38</v>
+      </c>
+      <c r="AE12" s="5" t="n">
+        <v>1043.92</v>
+      </c>
+      <c r="AF12" s="5" t="n">
+        <v>1086.52</v>
+      </c>
+      <c r="AG12" s="5" t="n">
+        <v>1011.959</v>
+      </c>
+      <c r="AH12" s="5" t="n">
+        <v>-0.63</v>
+      </c>
+      <c r="AI12" s="5" t="n">
+        <v>1150.4376</v>
+      </c>
+      <c r="AJ12" s="5" t="n">
+        <v>12.97</v>
+      </c>
+      <c r="AK12" s="5" t="n">
+        <v>1230.968232</v>
+      </c>
+      <c r="AL12" s="5" t="n">
+        <v>20.88</v>
+      </c>
+      <c r="AM12" s="5" t="n">
+        <v>1052.98</v>
+      </c>
+      <c r="AN12" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AO12" s="5" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="AP12" s="5" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="AQ12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR12" s="5" t="inlineStr"/>
+      <c r="AS12" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AT12" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="AA12" s="5" t="n">
-        <v>90</v>
-      </c>
-      <c r="AB12" s="5" t="n">
-        <v>91</v>
-      </c>
-      <c r="AC12" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="AD12" s="5" t="n">
-        <v>1065.22</v>
-      </c>
-      <c r="AE12" s="5" t="n">
-        <v>1018.38</v>
-      </c>
-      <c r="AF12" s="5" t="n">
-        <v>1043.92</v>
-      </c>
-      <c r="AG12" s="5" t="n">
-        <v>1086.52</v>
-      </c>
-      <c r="AH12" s="5" t="n">
-        <v>1011.959</v>
-      </c>
-      <c r="AI12" s="5" t="n">
-        <v>-0.63</v>
-      </c>
-      <c r="AJ12" s="5" t="n">
-        <v>1150.4376</v>
-      </c>
-      <c r="AK12" s="5" t="n">
+      <c r="AU12" s="5" t="n">
         <v>12.97</v>
       </c>
-      <c r="AL12" s="5" t="n">
-        <v>1230.968232</v>
-      </c>
-      <c r="AM12" s="5" t="n">
-        <v>20.88</v>
-      </c>
-      <c r="AN12" s="5" t="n">
-        <v>1052.98</v>
-      </c>
-      <c r="AO12" s="5" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AP12" s="5" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="AQ12" s="5" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="AR12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS12" s="5" t="inlineStr"/>
-      <c r="AT12" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AU12" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="AV12" s="5" t="n">
-        <v>12.97</v>
-      </c>
-      <c r="AW12" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-07 09:51</t>
+      <c r="AV12" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:01</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2570,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>R1_NEW</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -2649,143 +2588,138 @@
           <t>HOLD</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="H13" s="5" t="inlineStr"/>
       <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr"/>
-      <c r="K13" s="5" t="n">
+      <c r="J13" s="5" t="n">
         <v>10</v>
       </c>
+      <c r="K13" s="5" t="inlineStr"/>
       <c r="L13" s="5" t="inlineStr"/>
-      <c r="M13" s="5" t="inlineStr"/>
-      <c r="N13" s="5" t="n">
+      <c r="M13" s="5" t="n">
         <v>76.2</v>
       </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="P13" s="5" t="inlineStr">
-        <is>
           <t>🟢</t>
         </is>
       </c>
+      <c r="P13" s="5" t="n">
+        <v>52.9</v>
+      </c>
       <c r="Q13" s="5" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="R13" s="5" t="n">
         <v>-0.8</v>
       </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>crude +19.8% (rising) → +1.0pts · 15 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+        </is>
+      </c>
       <c r="S13" s="5" t="inlineStr">
         <is>
-          <t>crude +19.8% (rising) → +1.0pts · 15 insider Form 4 filings last 90d → +2.0pts (note: buy/sell parse pending)</t>
+          <t>🟢 BUY (Δ-2.0%) · Rank #10 · Conf 54% · momentum → · band HOLD · 91d left · → HOLD</t>
         </is>
       </c>
       <c r="T13" s="5" t="inlineStr">
         <is>
-          <t>🟢 BUY (Δ-2.0%) · Rank #10 · Conf 54% · momentum → · band HOLD · 91d left · → HOLD</t>
-        </is>
-      </c>
-      <c r="U13" s="5" t="inlineStr">
-        <is>
           <t>CRITICAL·DEEP_LOSS·-9.3% ≤ -8% · EXIT URGENT</t>
         </is>
       </c>
-      <c r="V13" s="5" t="n">
+      <c r="U13" s="5" t="n">
         <v>53.6</v>
       </c>
-      <c r="W13" s="5" t="inlineStr">
+      <c r="V13" s="5" t="inlineStr">
         <is>
           <t>Calibrated</t>
         </is>
       </c>
-      <c r="X13" s="5" t="n">
+      <c r="W13" s="5" t="n">
         <v>32.3</v>
       </c>
-      <c r="Y13" s="5" t="inlineStr"/>
+      <c r="X13" s="5" t="inlineStr"/>
+      <c r="Y13" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="Z13" s="5" t="n">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="AA13" s="5" t="n">
-        <v>90</v>
-      </c>
-      <c r="AB13" s="5" t="n">
         <v>91</v>
       </c>
-      <c r="AC13" s="5" t="inlineStr">
+      <c r="AB13" s="5" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
+      <c r="AC13" s="5" t="n">
+        <v>159.84</v>
+      </c>
       <c r="AD13" s="5" t="n">
-        <v>159.84</v>
+        <v>176.28</v>
       </c>
       <c r="AE13" s="5" t="n">
-        <v>176.28</v>
+        <v>156.64</v>
       </c>
       <c r="AF13" s="5" t="n">
-        <v>156.64</v>
+        <v>163.04</v>
       </c>
       <c r="AG13" s="5" t="n">
-        <v>163.04</v>
+        <v>151.848</v>
       </c>
       <c r="AH13" s="5" t="n">
-        <v>151.848</v>
+        <v>-13.86</v>
       </c>
       <c r="AI13" s="5" t="n">
-        <v>-13.86</v>
+        <v>172.6272</v>
       </c>
       <c r="AJ13" s="5" t="n">
-        <v>172.6272</v>
+        <v>-2.07</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>-2.07</v>
+        <v>184.711104</v>
       </c>
       <c r="AL13" s="5" t="n">
-        <v>184.711104</v>
+        <v>4.78</v>
       </c>
       <c r="AM13" s="5" t="n">
-        <v>4.78</v>
+        <v>181.45</v>
       </c>
       <c r="AN13" s="5" t="n">
-        <v>181.45</v>
+        <v>0.35</v>
       </c>
       <c r="AO13" s="5" t="n">
-        <v>0.35</v>
+        <v>-9.33</v>
       </c>
       <c r="AP13" s="5" t="n">
-        <v>-9.33</v>
+        <v>0</v>
       </c>
       <c r="AQ13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AR13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS13" s="5" t="inlineStr"/>
-      <c r="AT13" s="5" t="inlineStr">
+      <c r="AR13" s="5" t="inlineStr"/>
+      <c r="AS13" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AT13" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="AU13" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="AV13" s="5" t="n">
         <v>-2.07</v>
       </c>
-      <c r="AW13" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-07 09:51</t>
+      <c r="AV13" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-07 10:01</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AW13"/>
+  <autoFilter ref="A1:AV13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>